<commit_message>
docs: add 300 test cases for Selenium, ZAP, and API Performance
</commit_message>
<xml_diff>
--- a/CI_CD_Automation_Test_Report.xlsx
+++ b/CI_CD_Automation_Test_Report.xlsx
@@ -900,7 +900,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24 14:36:37</t>
+          <t>2026-07-25 09:52:46</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C5" s="31" t="inlineStr">
         <is>
-          <t>2026-07-24 14:36:38</t>
+          <t>2026-07-25 09:52:47</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>2026-07-24 14:36</t>
+          <t>2026-07-25 09:52</t>
         </is>
       </c>
       <c r="D18" s="5" t="n"/>
@@ -58015,7 +58015,7 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D15" s="31" t="inlineStr"/>

</xml_diff>